<commit_message>
Add qualitative theme diagram, participant matrix and joint display
</commit_message>
<xml_diff>
--- a/tez-calisma-ciktilari-2026-10-20/nitel-analiz-2026-10-22/NITEL-KODLAMA-VE-KANIT-TABLOLARI.xlsx
+++ b/tez-calisma-ciktilari-2026-10-20/nitel-analiz-2026-10-22/NITEL-KODLAMA-VE-KANIT-TABLOLARI.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soru_bazli_frekans" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoca_notlari" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dogrulanmis_alintilar" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Katilimci_karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nicel_nitel_ortak" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Kod_kitabi'!$A$1:$F$54</definedName>
@@ -25,6 +27,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Soru_bazli_frekans'!$A$1:$E$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hoca_notlari'!$A$1:$E$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Dogrulanmis_alintilar'!$A$1:$C$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Katilimci_karsilastirma'!$A$1:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Nicel_nitel_ortak'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2187,6 +2191,163 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bulgu alanı</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nicel bulgu</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nitel karşılık</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Birlikte okuma</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Yorum sınırı</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Problem çözme toplam puanı</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mevcut analizde N=40; ön 2.904, son 2.741; t(39)=2.372, p=.023, d_z=.375. Bu puanlamada düşük puan daha olumlu algıdır.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Dört görüşmede problem çözmeye katkı algısı vardır (P11). K1 problemi değiştirmeyi; K2, K3 ve K4 alternatif/çözüm üzerinde çalışmayı anlatır.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Genel yön bakımından uyum; deneyimlerde çeşitlilik.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Görüşmeler puan değişiminin nedeni veya bağımsız doğrulaması değildir. Dört görüşmeciyle 40 kişilik eşleşmiş örneklem arasında bireysel puan eşleştirmesi yapılmadı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Problem çözmede alt boyutlar</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mevcut analizde Güvenme: p&lt;.001; Kişisel Kontrol: p=.013; Yaklaşma–Kaçınma: p=.584. Düzeltilmemiş p değerleri.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>K1 çözüm bulamayınca problemi değiştirir (3-b). K2/K3 tasarım sorununda alternatif dener; K4 çözümün probleme yanıtını sorgular (3-b).</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Nitel veriler tek tip olmayan süreç deneyimleri ekler.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Bu anlatılar ölçek alt boyutlarıyla birebir eşitlenemez; anlamlı/anlamsız sonuçların nedenini kanıtladığı söylenemez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>İletişim toplam puanı</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mevcut analizde N=44; ön 3.832, son 3.910; t(43)=1.476, p=.147, d_z=.223. Anlamlı fark saptanmadı.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Dördü de rahat ifade ortamı anlatır (C01). K2, K3, K4 iletişim katkısı bildirir (C10); K2 büyüklükte temkinlidir (C12). K1’in 5-b yanıtı özgül beceri gelişimini adlandırmaz.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Veri türleri arasında görünüm farklılığı; rahat ortam ve gelişim ayrımı.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Olumlu deneyimler nicel anlamsız farkı geçersiz kılmaz. Önceden tanışıklık bağlam olarak anlatılabilir; farkın nedeninin bu olduğu gösterilmiş değildir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Öğrenme ve süreç yönetimi</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bu çalışma için eldeki iki ölçek, afet bilgisinde gecikmeli kalıcılığı, maliyeti veya ders içi beklemeyi doğrudan ölçmemektedir.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Dördü kalıcılık algısı bildirir (L02). Maliyet K1/K2/K4’te (L10); bekleme K2/K3’te (L12); planlama ve rehberlik önerileri R kodlarında yer alır.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Nitel verilerin kapsamı genişletici katkısı; doğrudan nicel eşdeğer yok.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Öğrenme kalıcılığı nesnel olarak ölçülmüş sayılmaz. Doğrudan nicel karşılığı olmayan bu deneyimler bulgu olarak korunur; yapay bir sayı veya ölçek puanı üretilmez.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -17138,4 +17299,242 @@
   <autoFilter ref="A1:C31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Boyut</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>K4</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Problem belirleme</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Zorlandı; özgünlük ve çözülebilirlik (1-a).</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Zorlanmadı; kısa araştırma yeterli oldu (1-a).</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Zorlandı; özgün problem/proje arayışı (1-a).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Zorlandı; yapılabilir proje seçimi (1-a).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Çözüm güçlüğüne yaklaşım</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Çözüm üretemeyince problemi değiştirdi (3-b).</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Tasarım güçlüğünde farklı yollar denedi (3-b).</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tasarım güçlüğünde vazgeçmeyip farklı yollar denedi (3-b).</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Çözümün probleme yanıtını sorgulayıp revize etti (3-b).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Fikir ifade etme ortamı</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Rahat ifade; kendi seçtiği grup (2-a).</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rahat ifade; kendi seçtiği grup (2-a).</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Rahat ifade; kendi seçtiği grup (2-a).</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Rahat ifade; önceden tanışıklık (2-a).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>İletişim becerisine katkı</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Özgül beceri adı yerine grup sürecini kolaylaştırma anlatımı (5-b).</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>İletişime katkı belirtti (5-a); belirli beceri katkısının büyüklüğünde temkinli (5-b).</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Çekingenliğine rağmen iletişim becerisinde güçlenme bildirdi (5-b).</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>İletişim ve birlikte çalışmaya katkı bildirdi (5-b).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Öğrenme algısı</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Araştırma, uygulama, ürün ve kalıcılık (4).</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Araştırma/uygulama, kalıcılık ve diğer sunumlardan öğrenme (4).</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Araştırarak/uygulayarak daha kalıcı öğrenme (4).</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Projede bilgiyi kullanma, kalıcılık ve diğer sunumlardan öğrenme (4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Başlıca güçlükler</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Yoruculuk/maliyet (6); serbest zamanın verimsiz kullanımı (7).</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Bekleme ve farklı ilerleme hızları (6); bütçe kısıtı (7).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Yoruculuk (6); öğretim elemanını/grupları bekleme (7).</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Uzun süren tasarım ve maliyet (6); farklı ilerleme hızları (7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Düzenleme önerileri</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Daha fazla süre ve planlı serbest zaman (7).</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Başlangıç örnekleri, bütçe/malzeme desteği (7); küçük gruplar (1-b).</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Bekleme sürelerini azaltıp ders zamanını verimli kullanma (7).</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Örnek ve rehberlik, özerkliği koruma, aşamaya uygun farklı görevler (7).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E8"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>